<commit_message>
Upgrade BUG-007 evidence: invalid signal value crashes the whole app
Not just a missing validation message — an unhandled client-side
RangeError unmounts the entire React app to a blank page, and permanently
breaks GET /api/offenders/{id} for the affected offender afterward.
Reproduced against two different seeded offenders today via automation.
</commit_message>
<xml_diff>
--- a/OffenderWatch_Tests.xlsx
+++ b/OffenderWatch_Tests.xlsx
@@ -8060,7 +8060,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Invalid manual location input fails without clear validation feedback</t>
+          <t>Invalid location signal value crashes the entire app (not just a validation gap)</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -8087,7 +8087,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>The operation/application fails or crashes without a clear validation message.</t>
+          <t>The client throws an unhandled RangeError ("Invalid count value: -1") and the whole React app unmounts to a blank white page. The offender the invalid point was submitted against is then permanently broken: GET /api/offenders/{id} returns HTTP 200 with an empty body from then on, for that offender specifically, with no way to recover it via the API (no delete-location endpoint). Reproduced twice independently today against two different seeded offenders (id=10 "Amar", then id=3 "Peretz") after submitting signal=6 through the Add Location form.</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
@@ -8097,7 +8097,7 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>UI error handling / API validation</t>
+          <t>UI (unhandled client-side exception) -- likely a bar/star rendering helper doing something like repeat(5 - signal) that goes negative when signal &gt; 5</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -16662,110 +16662,108 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>Automation — UI (Playwright)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>UI scenarios automated</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="0" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>UI passed</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="0" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>UI failed (confirmed defects)</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="0" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Automation — API (pytest + requests)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>API scenarios automated</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="0" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>API passed</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>API failed (confirmed defects)</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="0" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>Total confirmed defects (incl. BUG-016, BUG-017 found via automation)</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="0" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="11">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>Defects by severity</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>High: 15, Medium: 2, Low: 0</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="11">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Defect status</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>All 17 Open (0 fixed/retest)</t>
         </is>

</xml_diff>